<commit_message>
Day 07: RAND, ROUND, INT, TRUNC, LARGE and SMALL
</commit_message>
<xml_diff>
--- a/Excel/Day 05/Excel-Practice-(Day-05).xlsx
+++ b/Excel/Day 05/Excel-Practice-(Day-05).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analyst\Excel\Day 05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F16DB1B-6B03-4243-AC25-4BF6D091D6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AC07A31-4787-4B24-A47B-F6F5E004D98F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="678" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11835" tabRatio="678" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -34,6 +34,7 @@
     <definedName name="Slicer_Region">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
@@ -3901,6 +3902,12 @@
     <xf numFmtId="14" fontId="11" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3976,164 +3983,12 @@
     <xf numFmtId="0" fontId="21" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="58">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="4" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4936,6 +4791,152 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="4" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -5869,15 +5870,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="57" dataDxfId="55" headerRowBorderDxfId="56" tableBorderDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40">
   <autoFilter ref="A1:F38" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="53" totalsRowDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="51" totalsRowDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="49" totalsRowDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="47" totalsRowDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="45" totalsRowDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="43" totalsRowDxfId="42">
+    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
       <totalsRowFormula>SUM(F2:F38)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -18597,22 +18598,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="4:29" x14ac:dyDescent="0.25">
-      <c r="D1" s="192" t="s">
+      <c r="D1" s="194" t="s">
         <v>541</v>
       </c>
-      <c r="E1" s="193"/>
-      <c r="F1" s="193"/>
-      <c r="G1" s="193"/>
-      <c r="H1" s="193"/>
-      <c r="I1" s="193"/>
-      <c r="X1" s="194" t="s">
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
+      <c r="G1" s="195"/>
+      <c r="H1" s="195"/>
+      <c r="I1" s="195"/>
+      <c r="X1" s="196" t="s">
         <v>542</v>
       </c>
-      <c r="Y1" s="195"/>
-      <c r="Z1" s="195"/>
-      <c r="AA1" s="195"/>
-      <c r="AB1" s="195"/>
-      <c r="AC1" s="196"/>
+      <c r="Y1" s="197"/>
+      <c r="Z1" s="197"/>
+      <c r="AA1" s="197"/>
+      <c r="AB1" s="197"/>
+      <c r="AC1" s="198"/>
     </row>
     <row r="2" spans="4:29" x14ac:dyDescent="0.25">
       <c r="D2" s="106" t="s">
@@ -18633,29 +18634,29 @@
       <c r="I2" s="106" t="s">
         <v>537</v>
       </c>
-      <c r="K2" s="194" t="s">
+      <c r="K2" s="196" t="s">
         <v>543</v>
       </c>
-      <c r="L2" s="195"/>
-      <c r="M2" s="195"/>
-      <c r="N2" s="195"/>
-      <c r="O2" s="195"/>
-      <c r="P2" s="195"/>
-      <c r="Q2" s="195"/>
-      <c r="R2" s="195"/>
-      <c r="S2" s="195"/>
-      <c r="T2" s="195"/>
-      <c r="U2" s="195"/>
-      <c r="V2" s="196"/>
-      <c r="X2" s="192" t="str">
+      <c r="L2" s="197"/>
+      <c r="M2" s="197"/>
+      <c r="N2" s="197"/>
+      <c r="O2" s="197"/>
+      <c r="P2" s="197"/>
+      <c r="Q2" s="197"/>
+      <c r="R2" s="197"/>
+      <c r="S2" s="197"/>
+      <c r="T2" s="197"/>
+      <c r="U2" s="197"/>
+      <c r="V2" s="198"/>
+      <c r="X2" s="194" t="str">
         <f t="shared" ref="X2:X17" si="0">D1</f>
         <v>OPERATIONS</v>
       </c>
-      <c r="Y2" s="193"/>
-      <c r="Z2" s="193"/>
-      <c r="AA2" s="193"/>
-      <c r="AB2" s="193"/>
-      <c r="AC2" s="193"/>
+      <c r="Y2" s="195"/>
+      <c r="Z2" s="195"/>
+      <c r="AA2" s="195"/>
+      <c r="AB2" s="195"/>
+      <c r="AC2" s="195"/>
     </row>
     <row r="3" spans="4:29" x14ac:dyDescent="0.25">
       <c r="D3" s="105" t="s">
@@ -18672,7 +18673,7 @@
       </c>
       <c r="H3" s="135">
         <f t="shared" ref="H3:H16" ca="1" si="1">(RANDBETWEEN(10,50))/100</f>
-        <v>0.18</v>
+        <v>0.38</v>
       </c>
       <c r="I3" s="105">
         <v>100</v>
@@ -18717,7 +18718,7 @@
       </c>
       <c r="H4" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="X4" s="105" t="str">
         <f t="shared" si="0"/>
@@ -18737,7 +18738,7 @@
       </c>
       <c r="AB4" s="135">
         <f t="shared" ca="1" si="2"/>
-        <v>0.18</v>
+        <v>0.38</v>
       </c>
       <c r="AC4" s="105">
         <f t="shared" si="2"/>
@@ -18759,7 +18760,7 @@
       </c>
       <c r="H5" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.28999999999999998</v>
+        <v>0.17</v>
       </c>
       <c r="X5" s="105" t="str">
         <f t="shared" si="0"/>
@@ -18779,7 +18780,7 @@
       </c>
       <c r="AB5" s="135">
         <f t="shared" ref="AB5:AB17" ca="1" si="6">H4</f>
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="6" spans="4:29" x14ac:dyDescent="0.25">
@@ -18797,20 +18798,20 @@
       </c>
       <c r="H6" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.41</v>
-      </c>
-      <c r="L6" s="194" t="s">
+        <v>0.11</v>
+      </c>
+      <c r="L6" s="196" t="s">
         <v>540</v>
       </c>
-      <c r="M6" s="195"/>
-      <c r="N6" s="195"/>
-      <c r="O6" s="195"/>
-      <c r="P6" s="195"/>
-      <c r="Q6" s="195"/>
-      <c r="R6" s="195"/>
-      <c r="S6" s="195"/>
-      <c r="T6" s="195"/>
-      <c r="U6" s="196"/>
+      <c r="M6" s="197"/>
+      <c r="N6" s="197"/>
+      <c r="O6" s="197"/>
+      <c r="P6" s="197"/>
+      <c r="Q6" s="197"/>
+      <c r="R6" s="197"/>
+      <c r="S6" s="197"/>
+      <c r="T6" s="197"/>
+      <c r="U6" s="198"/>
       <c r="X6" s="105" t="str">
         <f t="shared" si="0"/>
         <v>Muhammad Hamza</v>
@@ -18829,7 +18830,7 @@
       </c>
       <c r="AB6" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.28999999999999998</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="7" spans="4:29" x14ac:dyDescent="0.25">
@@ -18847,7 +18848,7 @@
       </c>
       <c r="H7" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.36</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="X7" s="105" t="str">
         <f t="shared" si="0"/>
@@ -18867,7 +18868,7 @@
       </c>
       <c r="AB7" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.41</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="8" spans="4:29" x14ac:dyDescent="0.25">
@@ -18885,7 +18886,7 @@
       </c>
       <c r="H8" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.12</v>
+        <v>0.34</v>
       </c>
       <c r="M8" s="105">
         <v>137196</v>
@@ -18911,7 +18912,7 @@
       </c>
       <c r="AB8" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.36</v>
+        <v>0.28999999999999998</v>
       </c>
     </row>
     <row r="9" spans="4:29" x14ac:dyDescent="0.25">
@@ -18929,7 +18930,7 @@
       </c>
       <c r="H9" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.22</v>
+        <v>0.49</v>
       </c>
       <c r="M9" s="105">
         <v>64256</v>
@@ -18953,7 +18954,7 @@
       </c>
       <c r="AB9" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.12</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="10" spans="4:29" x14ac:dyDescent="0.25">
@@ -18971,7 +18972,7 @@
       </c>
       <c r="H10" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34</v>
+        <v>0.27</v>
       </c>
       <c r="M10" s="105">
         <v>137080</v>
@@ -18997,7 +18998,7 @@
       </c>
       <c r="AB10" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.22</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="11" spans="4:29" x14ac:dyDescent="0.25">
@@ -19015,7 +19016,7 @@
       </c>
       <c r="H11" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.42</v>
+        <v>0.5</v>
       </c>
       <c r="M11" s="105">
         <v>95302</v>
@@ -19041,7 +19042,7 @@
       </c>
       <c r="AB11" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.34</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="12" spans="4:29" x14ac:dyDescent="0.25">
@@ -19059,7 +19060,7 @@
       </c>
       <c r="H12" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.28000000000000003</v>
+        <v>0.34</v>
       </c>
       <c r="M12" s="105">
         <v>68657</v>
@@ -19085,7 +19086,7 @@
       </c>
       <c r="AB12" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.42</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="13" spans="4:29" x14ac:dyDescent="0.25">
@@ -19103,7 +19104,7 @@
       </c>
       <c r="H13" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="M13" s="105">
         <v>66062</v>
@@ -19129,7 +19130,7 @@
       </c>
       <c r="AB13" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.28000000000000003</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="14" spans="4:29" x14ac:dyDescent="0.25">
@@ -19147,7 +19148,7 @@
       </c>
       <c r="H14" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="M14" s="105">
         <v>98878</v>
@@ -19173,7 +19174,7 @@
       </c>
       <c r="AB14" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="15" spans="4:29" x14ac:dyDescent="0.25">
@@ -19191,7 +19192,7 @@
       </c>
       <c r="H15" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.14000000000000001</v>
+        <v>0.34</v>
       </c>
       <c r="M15" s="105">
         <v>40851</v>
@@ -19217,7 +19218,7 @@
       </c>
       <c r="AB15" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="16" spans="4:29" x14ac:dyDescent="0.25">
@@ -19235,7 +19236,7 @@
       </c>
       <c r="H16" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.3</v>
+        <v>0.49</v>
       </c>
       <c r="M16" s="105"/>
       <c r="N16" s="105"/>
@@ -19257,7 +19258,7 @@
       </c>
       <c r="AB16" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.14000000000000001</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="17" spans="4:28" x14ac:dyDescent="0.25">
@@ -19286,7 +19287,7 @@
       </c>
       <c r="AB17" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.3</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="18" spans="4:28" x14ac:dyDescent="0.25">
@@ -19334,31 +19335,31 @@
       </c>
     </row>
     <row r="29" spans="4:28" x14ac:dyDescent="0.25">
-      <c r="D29" s="193" t="s">
+      <c r="D29" s="195" t="s">
         <v>538</v>
       </c>
-      <c r="E29" s="193"/>
-      <c r="F29" s="193"/>
-      <c r="G29" s="193"/>
-      <c r="H29" s="193"/>
-      <c r="I29" s="193"/>
-      <c r="J29" s="193"/>
-      <c r="K29" s="193"/>
-      <c r="L29" s="193"/>
-      <c r="M29" s="193"/>
-      <c r="N29" s="193"/>
-      <c r="O29" s="193"/>
-      <c r="P29" s="193"/>
-      <c r="Q29" s="193"/>
-      <c r="R29" s="193"/>
-      <c r="U29" s="194" t="s">
+      <c r="E29" s="195"/>
+      <c r="F29" s="195"/>
+      <c r="G29" s="195"/>
+      <c r="H29" s="195"/>
+      <c r="I29" s="195"/>
+      <c r="J29" s="195"/>
+      <c r="K29" s="195"/>
+      <c r="L29" s="195"/>
+      <c r="M29" s="195"/>
+      <c r="N29" s="195"/>
+      <c r="O29" s="195"/>
+      <c r="P29" s="195"/>
+      <c r="Q29" s="195"/>
+      <c r="R29" s="195"/>
+      <c r="U29" s="196" t="s">
         <v>539</v>
       </c>
-      <c r="V29" s="195"/>
-      <c r="W29" s="195"/>
-      <c r="X29" s="195"/>
-      <c r="Y29" s="195"/>
-      <c r="Z29" s="196"/>
+      <c r="V29" s="197"/>
+      <c r="W29" s="197"/>
+      <c r="X29" s="197"/>
+      <c r="Y29" s="197"/>
+      <c r="Z29" s="198"/>
     </row>
     <row r="30" spans="4:28" x14ac:dyDescent="0.25">
       <c r="D30" s="106" t="s">
@@ -19893,38 +19894,38 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A4" s="197" t="s">
+      <c r="A4" s="199" t="s">
         <v>545</v>
       </c>
-      <c r="B4" s="198"/>
-      <c r="C4" s="198"/>
-      <c r="D4" s="198"/>
-      <c r="E4" s="198"/>
-      <c r="F4" s="198"/>
-      <c r="H4" s="197" t="s">
+      <c r="B4" s="200"/>
+      <c r="C4" s="200"/>
+      <c r="D4" s="200"/>
+      <c r="E4" s="200"/>
+      <c r="F4" s="200"/>
+      <c r="H4" s="199" t="s">
         <v>546</v>
       </c>
-      <c r="I4" s="198"/>
-      <c r="J4" s="198"/>
-      <c r="K4" s="198"/>
-      <c r="L4" s="198"/>
-      <c r="M4" s="198"/>
-      <c r="P4" s="197" t="s">
+      <c r="I4" s="200"/>
+      <c r="J4" s="200"/>
+      <c r="K4" s="200"/>
+      <c r="L4" s="200"/>
+      <c r="M4" s="200"/>
+      <c r="P4" s="199" t="s">
         <v>548</v>
       </c>
-      <c r="Q4" s="198"/>
-      <c r="R4" s="198"/>
-      <c r="S4" s="198"/>
-      <c r="T4" s="198"/>
-      <c r="U4" s="198"/>
-      <c r="W4" s="197" t="s">
+      <c r="Q4" s="200"/>
+      <c r="R4" s="200"/>
+      <c r="S4" s="200"/>
+      <c r="T4" s="200"/>
+      <c r="U4" s="200"/>
+      <c r="W4" s="199" t="s">
         <v>547</v>
       </c>
-      <c r="X4" s="198"/>
-      <c r="Y4" s="198"/>
-      <c r="Z4" s="198"/>
-      <c r="AA4" s="198"/>
-      <c r="AB4" s="198"/>
+      <c r="X4" s="200"/>
+      <c r="Y4" s="200"/>
+      <c r="Z4" s="200"/>
+      <c r="AA4" s="200"/>
+      <c r="AB4" s="200"/>
     </row>
     <row r="5" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
@@ -22393,22 +22394,22 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="199" t="s">
+      <c r="B3" s="201" t="s">
         <v>553</v>
       </c>
-      <c r="C3" s="199"/>
-      <c r="D3" s="199"/>
-      <c r="E3" s="199"/>
-      <c r="F3" s="199"/>
-      <c r="G3" s="200">
+      <c r="C3" s="201"/>
+      <c r="D3" s="201"/>
+      <c r="E3" s="201"/>
+      <c r="F3" s="201"/>
+      <c r="G3" s="202">
         <v>400</v>
       </c>
-      <c r="H3" s="200"/>
-      <c r="I3" s="200"/>
-      <c r="J3" s="200"/>
-      <c r="K3" s="200"/>
-      <c r="L3" s="200"/>
-      <c r="M3" s="200"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
+      <c r="J3" s="202"/>
+      <c r="K3" s="202"/>
+      <c r="L3" s="202"/>
+      <c r="M3" s="202"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="137" t="s">
@@ -23109,18 +23110,18 @@
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B25" s="199" t="s">
+      <c r="B25" s="201" t="s">
         <v>553</v>
       </c>
-      <c r="C25" s="199"/>
-      <c r="D25" s="199"/>
-      <c r="E25" s="199"/>
-      <c r="F25" s="199"/>
-      <c r="G25" s="201">
+      <c r="C25" s="201"/>
+      <c r="D25" s="201"/>
+      <c r="E25" s="201"/>
+      <c r="F25" s="201"/>
+      <c r="G25" s="203">
         <v>400</v>
       </c>
-      <c r="H25" s="202"/>
-      <c r="I25" s="202"/>
+      <c r="H25" s="204"/>
+      <c r="I25" s="204"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" s="137" t="s">
@@ -24014,14 +24015,14 @@
       </c>
     </row>
     <row r="24" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="203" t="s">
+      <c r="B24" s="205" t="s">
         <v>734</v>
       </c>
-      <c r="C24" s="204"/>
-      <c r="D24" s="204"/>
-      <c r="E24" s="204"/>
-      <c r="F24" s="204"/>
-      <c r="G24" s="205"/>
+      <c r="C24" s="206"/>
+      <c r="D24" s="206"/>
+      <c r="E24" s="206"/>
+      <c r="F24" s="206"/>
+      <c r="G24" s="207"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -24063,19 +24064,19 @@
   <sheetData>
     <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="206" t="s">
+      <c r="B2" s="208" t="s">
         <v>564</v>
       </c>
-      <c r="C2" s="207"/>
+      <c r="C2" s="209"/>
       <c r="D2" s="145"/>
-      <c r="E2" s="206" t="s">
+      <c r="E2" s="208" t="s">
         <v>568</v>
       </c>
-      <c r="F2" s="207"/>
-      <c r="H2" s="206" t="s">
+      <c r="F2" s="209"/>
+      <c r="H2" s="208" t="s">
         <v>572</v>
       </c>
-      <c r="I2" s="207"/>
+      <c r="I2" s="209"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="148" t="s">
@@ -24316,14 +24317,14 @@
     </row>
     <row r="15" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="206" t="s">
+      <c r="B16" s="208" t="s">
         <v>687</v>
       </c>
-      <c r="C16" s="207"/>
-      <c r="E16" s="206" t="s">
+      <c r="C16" s="209"/>
+      <c r="E16" s="208" t="s">
         <v>580</v>
       </c>
-      <c r="F16" s="207"/>
+      <c r="F16" s="209"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="148" t="s">
@@ -24481,18 +24482,18 @@
     </row>
     <row r="31" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="206" t="s">
+      <c r="B32" s="208" t="s">
         <v>588</v>
       </c>
-      <c r="C32" s="207"/>
-      <c r="E32" s="206" t="s">
+      <c r="C32" s="209"/>
+      <c r="E32" s="208" t="s">
         <v>584</v>
       </c>
-      <c r="F32" s="207"/>
-      <c r="H32" s="206" t="s">
+      <c r="F32" s="209"/>
+      <c r="H32" s="208" t="s">
         <v>592</v>
       </c>
-      <c r="I32" s="207"/>
+      <c r="I32" s="209"/>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B33" s="148" t="s">
@@ -24722,39 +24723,39 @@
       </c>
     </row>
     <row r="45" spans="2:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="208" t="s">
+      <c r="B45" s="210" t="s">
         <v>732</v>
       </c>
-      <c r="C45" s="208"/>
-      <c r="D45" s="208"/>
+      <c r="C45" s="210"/>
+      <c r="D45" s="210"/>
       <c r="E45" s="170"/>
       <c r="F45" s="170"/>
-      <c r="G45" s="208" t="s">
+      <c r="G45" s="210" t="s">
         <v>719</v>
       </c>
-      <c r="H45" s="208"/>
-      <c r="I45" s="208"/>
+      <c r="H45" s="210"/>
+      <c r="I45" s="210"/>
       <c r="J45" s="170"/>
-      <c r="K45" s="208" t="s">
+      <c r="K45" s="210" t="s">
         <v>707</v>
       </c>
-      <c r="L45" s="208"/>
-      <c r="M45" s="208"/>
-      <c r="O45" s="208" t="s">
+      <c r="L45" s="210"/>
+      <c r="M45" s="210"/>
+      <c r="O45" s="210" t="s">
         <v>730</v>
       </c>
-      <c r="P45" s="208"/>
-      <c r="Q45" s="208"/>
-      <c r="S45" s="208" t="s">
+      <c r="P45" s="210"/>
+      <c r="Q45" s="210"/>
+      <c r="S45" s="210" t="s">
         <v>731</v>
       </c>
-      <c r="T45" s="208"/>
-      <c r="U45" s="208"/>
-      <c r="W45" s="208" t="s">
+      <c r="T45" s="210"/>
+      <c r="U45" s="210"/>
+      <c r="W45" s="210" t="s">
         <v>733</v>
       </c>
-      <c r="X45" s="208"/>
-      <c r="Y45" s="208"/>
+      <c r="X45" s="210"/>
+      <c r="Y45" s="210"/>
     </row>
     <row r="46" spans="2:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="167" t="s">
@@ -25441,11 +25442,11 @@
       <c r="D59" s="170"/>
       <c r="E59" s="170"/>
       <c r="F59" s="170"/>
-      <c r="G59" s="208" t="s">
+      <c r="G59" s="210" t="s">
         <v>735</v>
       </c>
-      <c r="H59" s="208"/>
-      <c r="I59" s="208"/>
+      <c r="H59" s="210"/>
+      <c r="I59" s="210"/>
       <c r="J59" s="170"/>
       <c r="K59" s="170"/>
       <c r="L59" s="170"/>
@@ -25552,22 +25553,22 @@
     </row>
     <row r="74" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="75" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B75" s="206" t="s">
+      <c r="B75" s="208" t="s">
         <v>738</v>
       </c>
-      <c r="C75" s="207"/>
-      <c r="E75" s="206" t="s">
+      <c r="C75" s="209"/>
+      <c r="E75" s="208" t="s">
         <v>741</v>
       </c>
-      <c r="F75" s="207"/>
-      <c r="H75" s="206" t="s">
+      <c r="F75" s="209"/>
+      <c r="H75" s="208" t="s">
         <v>740</v>
       </c>
-      <c r="I75" s="207"/>
-      <c r="K75" s="206" t="s">
+      <c r="I75" s="209"/>
+      <c r="K75" s="208" t="s">
         <v>742</v>
       </c>
-      <c r="L75" s="207"/>
+      <c r="L75" s="209"/>
     </row>
     <row r="76" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B76" s="148" t="s">
@@ -25867,10 +25868,10 @@
     </row>
     <row r="89" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="90" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="206" t="s">
+      <c r="B90" s="208" t="s">
         <v>628</v>
       </c>
-      <c r="C90" s="207"/>
+      <c r="C90" s="209"/>
     </row>
     <row r="91" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B91" s="148" t="s">
@@ -25882,14 +25883,14 @@
       <c r="D91" s="148" t="s">
         <v>745</v>
       </c>
-      <c r="F91" s="206" t="s">
+      <c r="F91" s="208" t="s">
         <v>746</v>
       </c>
-      <c r="G91" s="207"/>
-      <c r="I91" s="206" t="s">
+      <c r="G91" s="209"/>
+      <c r="I91" s="208" t="s">
         <v>748</v>
       </c>
-      <c r="J91" s="207"/>
+      <c r="J91" s="209"/>
     </row>
     <row r="92" spans="2:12" ht="30" x14ac:dyDescent="0.25">
       <c r="B92" s="183">
@@ -25903,14 +25904,14 @@
         <f>TEXT(B92,"MMMM")</f>
         <v>October</v>
       </c>
-      <c r="F92" s="209" t="s">
+      <c r="F92" s="184" t="s">
         <v>747</v>
       </c>
       <c r="G92" s="149">
         <f>VALUE(F92)</f>
         <v>12345</v>
       </c>
-      <c r="I92" s="210" t="s">
+      <c r="I92" s="185" t="s">
         <v>749</v>
       </c>
       <c r="J92" s="149" t="str">
@@ -25923,7 +25924,7 @@
         <v>46310</v>
       </c>
       <c r="C93" s="149" t="str">
-        <f t="shared" ref="C93:D100" si="16">TEXT(B93,"DDDD")</f>
+        <f t="shared" ref="C93:C100" si="16">TEXT(B93,"DDDD")</f>
         <v>Thursday</v>
       </c>
       <c r="D93" s="149" t="str">
@@ -25982,14 +25983,14 @@
         <f t="shared" si="17"/>
         <v>October</v>
       </c>
-      <c r="F97" s="206" t="s">
+      <c r="F97" s="208" t="s">
         <v>637</v>
       </c>
-      <c r="G97" s="207"/>
-      <c r="I97" s="206" t="s">
+      <c r="G97" s="209"/>
+      <c r="I97" s="208" t="s">
         <v>641</v>
       </c>
-      <c r="J97" s="207"/>
+      <c r="J97" s="209"/>
     </row>
     <row r="98" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B98" s="183">
@@ -26003,14 +26004,14 @@
         <f t="shared" si="17"/>
         <v>October</v>
       </c>
-      <c r="F98" s="209" t="s">
+      <c r="F98" s="184" t="s">
         <v>750</v>
       </c>
       <c r="G98" s="149" t="str">
         <f>CHAR(F98)</f>
         <v>A</v>
       </c>
-      <c r="I98" s="209" t="s">
+      <c r="I98" s="184" t="s">
         <v>751</v>
       </c>
       <c r="J98" s="149" t="str">
@@ -26046,17 +26047,20 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="H75:I75"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="I91:J91"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="E16:F16"/>
     <mergeCell ref="F97:G97"/>
     <mergeCell ref="I97:J97"/>
     <mergeCell ref="W45:Y45"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="H32:I32"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="E16:F16"/>
     <mergeCell ref="B45:D45"/>
     <mergeCell ref="G45:I45"/>
     <mergeCell ref="K45:M45"/>
@@ -26067,9 +26071,6 @@
     <mergeCell ref="B75:C75"/>
     <mergeCell ref="E75:F75"/>
     <mergeCell ref="K75:L75"/>
-    <mergeCell ref="H75:I75"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="I91:J91"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -28531,11 +28532,11 @@
       </c>
       <c r="D2" s="25">
         <f t="shared" ref="C2:F15" ca="1" si="0">RANDBETWEEN(0,100)</f>
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="E2" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="F2" s="25"/>
       <c r="G2" s="28">
@@ -28557,16 +28558,16 @@
       </c>
       <c r="C3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="D3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="E3" s="25"/>
       <c r="F3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G3" s="28">
         <f t="shared" ref="G3:G15" ca="1" si="1">COUNT(C3:F3)</f>
@@ -28588,11 +28589,11 @@
       <c r="C4" s="25"/>
       <c r="D4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>36</v>
+        <v>98</v>
       </c>
       <c r="E4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>71</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="28">
@@ -28614,16 +28615,16 @@
       </c>
       <c r="C5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="D5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E5" s="25"/>
       <c r="F5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G5" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28644,16 +28645,16 @@
       </c>
       <c r="C6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="D6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="E6" s="25"/>
       <c r="F6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="G6" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28675,15 +28676,15 @@
       <c r="C7" s="25"/>
       <c r="D7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="E7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="G7" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28704,7 +28705,7 @@
       </c>
       <c r="C8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>468</v>
@@ -28714,7 +28715,7 @@
       </c>
       <c r="F8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="G8" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28735,19 +28736,19 @@
       </c>
       <c r="C9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="D9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="E9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="F9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="G9" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28768,12 +28769,12 @@
       </c>
       <c r="C10" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D10" s="25"/>
       <c r="E10" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="F10" s="25"/>
       <c r="G10" s="28">
@@ -28795,19 +28796,19 @@
       </c>
       <c r="C11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>11</v>
+        <v>72</v>
       </c>
       <c r="D11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="E11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="F11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="G11" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28828,15 +28829,15 @@
       </c>
       <c r="C12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="D12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="E12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F12" s="25"/>
       <c r="G12" s="28">
@@ -28858,16 +28859,16 @@
       </c>
       <c r="C13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="D13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="G13" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28888,18 +28889,18 @@
       </c>
       <c r="C14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>45</v>
+        <v>83</v>
       </c>
       <c r="D14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>468</v>
       </c>
       <c r="F14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="G14" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28924,7 +28925,7 @@
       <c r="D15" s="27"/>
       <c r="E15" s="27">
         <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="F15" s="27" t="s">
         <v>468</v>
@@ -33361,54 +33362,54 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E51">
-    <cfRule type="cellIs" dxfId="41" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="44" operator="equal">
       <formula>20000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="45" operator="between">
+    <cfRule type="cellIs" dxfId="56" priority="45" operator="between">
       <formula>50000</formula>
       <formula>100000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="46" operator="between">
+    <cfRule type="cellIs" dxfId="55" priority="46" operator="between">
       <formula>"Rs. 65,984"</formula>
       <formula>"Rs. 121,395"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="47" operator="lessThan">
+    <cfRule type="cellIs" dxfId="54" priority="47" operator="lessThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="48" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="53" priority="48" operator="greaterThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="49" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="52" priority="49" operator="greaterThan">
       <formula>"Rs. 93,689"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B53">
-    <cfRule type="containsText" dxfId="35" priority="43" operator="containsText" text="Ayesha khan">
+    <cfRule type="containsText" dxfId="51" priority="43" operator="containsText" text="Ayesha khan">
       <formula>NOT(ISERROR(SEARCH("Ayesha khan",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A53">
-    <cfRule type="timePeriod" dxfId="34" priority="41" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="50" priority="41" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="33" priority="42" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="49" priority="42" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A53">
-    <cfRule type="timePeriod" dxfId="32" priority="38" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="48" priority="38" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A2,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A2,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="31" priority="39" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="47" priority="39" timePeriod="yesterday">
       <formula>FLOOR(A2,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="30" priority="40" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="46" priority="40" timePeriod="today">
       <formula>FLOOR(A2,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="uniqueValues" dxfId="29" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="37"/>
+    <cfRule type="uniqueValues" dxfId="45" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E55:E105">
     <cfRule type="dataBar" priority="18">
@@ -35624,13 +35625,13 @@
     </row>
     <row r="58" spans="3:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="59" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C59" s="184" t="s">
+      <c r="C59" s="186" t="s">
         <v>528</v>
       </c>
-      <c r="D59" s="185"/>
-      <c r="E59" s="185"/>
-      <c r="F59" s="185"/>
-      <c r="G59" s="185"/>
+      <c r="D59" s="187"/>
+      <c r="E59" s="187"/>
+      <c r="F59" s="187"/>
+      <c r="G59" s="187"/>
       <c r="H59" s="88"/>
     </row>
     <row r="60" spans="3:8" x14ac:dyDescent="0.25">
@@ -40930,40 +40931,40 @@
     </row>
     <row r="168" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="169" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A169" s="186" t="s">
+      <c r="A169" s="188" t="s">
         <v>534</v>
       </c>
-      <c r="B169" s="187"/>
-      <c r="C169" s="187"/>
-      <c r="D169" s="187"/>
-      <c r="E169" s="187"/>
-      <c r="F169" s="187"/>
-      <c r="G169" s="187"/>
-      <c r="H169" s="187"/>
-      <c r="I169" s="187"/>
-      <c r="J169" s="187"/>
-      <c r="K169" s="187"/>
-      <c r="L169" s="187"/>
-      <c r="M169" s="187"/>
-      <c r="N169" s="187"/>
-      <c r="O169" s="188"/>
+      <c r="B169" s="189"/>
+      <c r="C169" s="189"/>
+      <c r="D169" s="189"/>
+      <c r="E169" s="189"/>
+      <c r="F169" s="189"/>
+      <c r="G169" s="189"/>
+      <c r="H169" s="189"/>
+      <c r="I169" s="189"/>
+      <c r="J169" s="189"/>
+      <c r="K169" s="189"/>
+      <c r="L169" s="189"/>
+      <c r="M169" s="189"/>
+      <c r="N169" s="189"/>
+      <c r="O169" s="190"/>
     </row>
     <row r="170" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="189"/>
-      <c r="B170" s="190"/>
-      <c r="C170" s="190"/>
-      <c r="D170" s="190"/>
-      <c r="E170" s="190"/>
-      <c r="F170" s="190"/>
-      <c r="G170" s="190"/>
-      <c r="H170" s="190"/>
-      <c r="I170" s="190"/>
-      <c r="J170" s="190"/>
-      <c r="K170" s="190"/>
-      <c r="L170" s="190"/>
-      <c r="M170" s="190"/>
-      <c r="N170" s="190"/>
-      <c r="O170" s="191"/>
+      <c r="A170" s="191"/>
+      <c r="B170" s="192"/>
+      <c r="C170" s="192"/>
+      <c r="D170" s="192"/>
+      <c r="E170" s="192"/>
+      <c r="F170" s="192"/>
+      <c r="G170" s="192"/>
+      <c r="H170" s="192"/>
+      <c r="I170" s="192"/>
+      <c r="J170" s="192"/>
+      <c r="K170" s="192"/>
+      <c r="L170" s="192"/>
+      <c r="M170" s="192"/>
+      <c r="N170" s="192"/>
+      <c r="O170" s="193"/>
     </row>
     <row r="171" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A171" s="112"/>

</xml_diff>